<commit_message>
Migrate remaining 13 WKND adventure detail pages
Import all remaining adventure detail pages (beervana-portland,
climbing-new-zealand, colorado-rock-climbing, cycling-southern-utah,
cycling-tuscany, downhill-skiing-wyoming, gastronomic-marais-tour,
napa-wine-tasting, riverside-camping-australia, ski-touring-mont-blanc,
surf-camp-costa-rica, west-coast-cycling, whistler-mountain-biking),
bringing the adventure-detail template to all 16 URLs.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,7 +73,7 @@
     <t>adventures-listing</t>
   </si>
   <si>
-    <t>2026-07-23T10:43:12.588Z</t>
+    <t>2026-07-23T10:48:53.507Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -82,10 +82,19 @@
     <t>https://wknd.site/us/en/adventures.html</t>
   </si>
   <si>
+    <t>us/en/index.report.json</t>
+  </si>
+  <si>
+    <t>us/en/index</t>
+  </si>
+  <si>
+    <t>2026-07-23T13:34:29.830Z</t>
+  </si>
+  <si>
     <t>us/en/adventures/bali-surf-camp.report.json</t>
   </si>
   <si>
-    <t>["breadcrumb","hero","info-panel","tabs"]</t>
+    <t>["breadcrumb","carousel","info-panel","tabs"]</t>
   </si>
   <si>
     <t>us/en/adventures/bali-surf-camp</t>
@@ -94,7 +103,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-07-23T10:43:16.349Z</t>
+    <t>2026-07-23T14:49:54.433Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -103,13 +112,178 @@
     <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
   </si>
   <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:39:27.289Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:39:31.314Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:39:37.241Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:39:43.078Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:39:49.451Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:39:55.446Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:00.433Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:05.098Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:10.238Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:14.176Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:18.804Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/tahoe-skiing.report.json</t>
   </si>
   <si>
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-07-23T10:43:26.047Z</t>
+    <t>2026-07-23T14:50:05.561Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -118,13 +292,43 @@
     <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
   </si>
   <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:24.239Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-07-23T16:40:29.277Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/yosemite-backpacking.report.json</t>
   </si>
   <si>
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-07-23T10:43:20.906Z</t>
+    <t>2026-07-23T14:49:59.827Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -519,11 +723,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="39" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
@@ -613,77 +817,441 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>27</v>
-      </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="G5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>32</v>
-      </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
         <v>36</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>37</v>
       </c>
-      <c r="G6" t="s">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>38</v>
       </c>
-      <c r="H6" t="s">
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
         <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" t="s">
+        <v>75</v>
+      </c>
+      <c r="G14" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" t="s">
+        <v>91</v>
+      </c>
+      <c r="H17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" t="s">
+        <v>96</v>
+      </c>
+      <c r="H18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" t="s">
+        <v>100</v>
+      </c>
+      <c r="G19" t="s">
+        <v>101</v>
+      </c>
+      <c r="H19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" t="s">
+        <v>105</v>
+      </c>
+      <c r="G20" t="s">
+        <v>106</v>
+      </c>
+      <c r="H20" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix tabs parser to preserve headings and image captions
The tabs parser dropped H2/H3 section headings (filtered out as non-content
inside AEM's .aem-Grid wrapper) and image captions (span.cmp-image__title was
never collected). Allow H1-H6 through the grid filter and promote image
captions to italic paragraphs. Re-import all 16 adventure detail pages.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -103,7 +103,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-07-23T14:49:54.433Z</t>
+    <t>2026-07-23T16:57:37.007Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -118,7 +118,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-07-23T16:39:27.289Z</t>
+    <t>2026-07-23T16:57:52.664Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -133,7 +133,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-07-23T16:39:31.314Z</t>
+    <t>2026-07-23T16:57:58.808Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -148,7 +148,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-07-23T16:39:37.241Z</t>
+    <t>2026-07-23T16:58:02.547Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -163,7 +163,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-07-23T16:39:43.078Z</t>
+    <t>2026-07-23T16:58:08.523Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -178,7 +178,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-07-23T16:39:49.451Z</t>
+    <t>2026-07-23T16:58:14.054Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -193,7 +193,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-07-23T16:39:55.446Z</t>
+    <t>2026-07-23T16:58:17.706Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -208,7 +208,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:00.433Z</t>
+    <t>2026-07-23T16:58:22.754Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -223,7 +223,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:05.098Z</t>
+    <t>2026-07-23T16:58:28.017Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -238,7 +238,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:10.238Z</t>
+    <t>2026-07-23T16:58:32.369Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -253,7 +253,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:14.176Z</t>
+    <t>2026-07-23T16:58:37.013Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -268,7 +268,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:18.804Z</t>
+    <t>2026-07-23T16:58:40.961Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -283,7 +283,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-07-23T14:50:05.561Z</t>
+    <t>2026-07-23T16:57:48.375Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -298,7 +298,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:24.239Z</t>
+    <t>2026-07-23T16:58:45.064Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -313,7 +313,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-07-23T16:40:29.277Z</t>
+    <t>2026-07-23T16:58:49.604Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -328,7 +328,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-07-23T14:49:59.827Z</t>
+    <t>2026-07-23T16:57:42.236Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>

</xml_diff>

<commit_message>
Make adventures listing dynamic via query index
Rewrite adventure-filter to fetch /us/en/adventures/query-index.json at
runtime and build the filterable card grid from the adventure detail
child pages, instead of a static authored card list. Adds helix-query.yaml
indexing /us/en/adventures/** with a Category property, and injects a
Category metadata field into each detail page at import time.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="165">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,6 +61,27 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards-person","cards-person","cards-person","cards-person","cards-person","cards-person","cards-person"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>about-us</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:26:25.905Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
@@ -82,6 +103,27 @@
     <t>https://wknd.site/us/en/adventures.html</t>
   </si>
   <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faqs</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:21:41.008Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
     <t>us/en/index.report.json</t>
   </si>
   <si>
@@ -91,6 +133,36 @@
     <t>2026-07-23T13:34:29.830Z</t>
   </si>
   <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>["columns","columns","columns","cards"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>magazine-listing</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:21:37.075Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>us/en/about-us/index.report.json</t>
+  </si>
+  <si>
+    <t>us/en/about-us/index</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:33:38.135Z</t>
+  </si>
+  <si>
     <t>us/en/adventures/bali-surf-camp.report.json</t>
   </si>
   <si>
@@ -103,7 +175,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-07-23T16:57:37.007Z</t>
+    <t>2026-07-24T05:30:31.309Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -118,7 +190,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-07-23T16:57:52.664Z</t>
+    <t>2026-07-24T05:30:47.443Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -133,7 +205,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-07-23T16:57:58.808Z</t>
+    <t>2026-07-24T05:30:52.849Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -148,7 +220,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:02.547Z</t>
+    <t>2026-07-24T05:30:57.997Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -163,7 +235,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:08.523Z</t>
+    <t>2026-07-24T05:31:02.184Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -178,7 +250,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:14.054Z</t>
+    <t>2026-07-24T05:31:07.044Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -193,7 +265,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:17.706Z</t>
+    <t>2026-07-24T05:31:12.371Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -208,7 +280,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:22.754Z</t>
+    <t>2026-07-24T05:31:17.755Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -223,7 +295,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:28.017Z</t>
+    <t>2026-07-24T05:31:22.490Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -238,7 +310,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:32.369Z</t>
+    <t>2026-07-24T05:31:26.684Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -253,7 +325,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:37.013Z</t>
+    <t>2026-07-24T05:31:31.856Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -268,7 +340,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:40.961Z</t>
+    <t>2026-07-24T05:31:37.342Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -283,7 +355,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-07-23T16:57:48.375Z</t>
+    <t>2026-07-24T05:30:42.050Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -298,7 +370,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:45.064Z</t>
+    <t>2026-07-24T05:31:43.535Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -313,7 +385,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-07-23T16:58:49.604Z</t>
+    <t>2026-07-24T05:31:49.268Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -328,13 +400,112 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-07-23T16:57:42.236Z</t>
+    <t>2026-07-24T05:30:36.440Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs/index.report.json</t>
+  </si>
+  <si>
+    <t>us/en/faqs/index</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:33:34.156Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb","cards"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>magazine-article</t>
+  </si>
+  <si>
+    <t>2026-07-23T17:21:38.449Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-07-23T19:07:45.226Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/index.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/index</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:33:29.987Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:52:50.187Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:52:55.480Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-07-23T18:53:07.795Z</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/western-australia.html</t>
   </si>
 </sst>
 </file>
@@ -723,14 +894,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="46" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="7" max="7" width="33" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -817,441 +988,727 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="H8" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
         <v>53</v>
       </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>29</v>
-      </c>
       <c r="F10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H13" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G14" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G15" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H15" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G17" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F18" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G18" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H18" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F19" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G19" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="F20" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G20" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" t="s">
+        <v>114</v>
+      </c>
+      <c r="G21" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" t="s">
+        <v>120</v>
+      </c>
+      <c r="H22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" t="s">
+        <v>124</v>
+      </c>
+      <c r="G23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" t="s">
+        <v>128</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" t="s">
+        <v>129</v>
+      </c>
+      <c r="G24" t="s">
+        <v>130</v>
+      </c>
+      <c r="H24" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" t="s">
+        <v>134</v>
+      </c>
+      <c r="G25" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" t="s">
+        <v>136</v>
+      </c>
+      <c r="C26" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>138</v>
+      </c>
+      <c r="F26" t="s">
+        <v>139</v>
+      </c>
+      <c r="G26" t="s">
+        <v>140</v>
+      </c>
+      <c r="H26" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>138</v>
+      </c>
+      <c r="F27" t="s">
+        <v>144</v>
+      </c>
+      <c r="G27" t="s">
+        <v>145</v>
+      </c>
+      <c r="H27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>43</v>
+      </c>
+      <c r="F28" t="s">
+        <v>149</v>
+      </c>
+      <c r="G28" t="s">
+        <v>45</v>
+      </c>
+      <c r="H28" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" t="s">
+        <v>151</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>138</v>
+      </c>
+      <c r="F29" t="s">
+        <v>152</v>
+      </c>
+      <c r="G29" t="s">
+        <v>153</v>
+      </c>
+      <c r="H29" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>155</v>
+      </c>
+      <c r="B30" t="s">
+        <v>136</v>
+      </c>
+      <c r="C30" t="s">
+        <v>156</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>138</v>
+      </c>
+      <c r="F30" t="s">
+        <v>157</v>
+      </c>
+      <c r="G30" t="s">
+        <v>158</v>
+      </c>
+      <c r="H30" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>138</v>
+      </c>
+      <c r="F31" t="s">
+        <v>162</v>
+      </c>
+      <c r="G31" t="s">
+        <v>163</v>
+      </c>
+      <c r="H31" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>